<commit_message>
Layers 1-2: factor ingestion + 36mo flag (module 0); residuals, factor covariance, Ledoit-Wolf/factor-decomposition switch (module 1)
</commit_message>
<xml_diff>
--- a/asian_fx_vs_usd.xlsx
+++ b/asian_fx_vs_usd.xlsx
@@ -491,12 +491,12 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>Rate 2025-05-16</t>
+          <t>Rate 2025-06-14</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Rate 2026-05-16</t>
+          <t>Rate 2026-06-14</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
@@ -527,13 +527,13 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>145.613</v>
+        <v>143.194</v>
       </c>
       <c r="E2" s="3" t="n">
-        <v>158.731</v>
+        <v>160.13</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>0.0901</v>
+        <v>0.1183</v>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
@@ -558,13 +558,13 @@
         </is>
       </c>
       <c r="D3" s="3" t="n">
-        <v>7.2065</v>
+        <v>7.1928</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>6.8087</v>
+        <v>6.7755</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>-0.0552</v>
+        <v>-0.058</v>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
@@ -589,13 +589,13 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>85.4449</v>
+        <v>85.6884</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>95.955</v>
+        <v>95.76009999999999</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>0.123</v>
+        <v>0.1175</v>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
@@ -620,13 +620,13 @@
         </is>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1397.02</v>
+        <v>1349.79</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1497.76</v>
+        <v>1517.38</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0.0721</v>
+        <v>0.1242</v>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
@@ -651,17 +651,17 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>7.8054</v>
+        <v>7.8489</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>7.8293</v>
+        <v>7.8356</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>0.0031</v>
+        <v>-0.0017</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Weakened</t>
+          <t>Strengthened</t>
         </is>
       </c>
     </row>
@@ -682,17 +682,17 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1.2966</v>
+        <v>1.2782</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>1.2765</v>
+        <v>1.2841</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>-0.0155</v>
+        <v>0.0046</v>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Strengthened</t>
+          <t>Weakened</t>
         </is>
       </c>
     </row>
@@ -713,13 +713,13 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>30.167</v>
+        <v>29.5252</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>31.56</v>
+        <v>31.579</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>0.0462</v>
+        <v>0.0696</v>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
@@ -744,17 +744,17 @@
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>33.18</v>
+        <v>32.34</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>32.65</v>
+        <v>32.705</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>-0.016</v>
+        <v>0.0113</v>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Strengthened</t>
+          <t>Weakened</t>
         </is>
       </c>
     </row>
@@ -775,13 +775,13 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>4.28</v>
+        <v>4.2185</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>3.947</v>
+        <v>4.0644</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>-0.07780000000000001</v>
+        <v>-0.0365</v>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
@@ -806,13 +806,13 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>16511.8008</v>
+        <v>16164.5</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>17491</v>
+        <v>17921</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>0.0593</v>
+        <v>0.1087</v>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
@@ -837,13 +837,13 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>55.635</v>
+        <v>54.194</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>61.648</v>
+        <v>60.971</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>0.1081</v>
+        <v>0.1251</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
@@ -868,13 +868,13 @@
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>25920</v>
+        <v>26020</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>26350</v>
+        <v>26325</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>0.0166</v>
+        <v>0.0117</v>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
@@ -908,7 +908,7 @@
       </c>
       <c r="B1" s="7" t="inlineStr">
         <is>
-          <t>2025-05-16  →  2026-05-16</t>
+          <t>2025-06-14  →  2026-06-14</t>
         </is>
       </c>
     </row>
@@ -930,7 +930,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>MYR (-7.78%)</t>
+          <t>CNY (-5.80%)</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>INR (+12.30%)</t>
+          <t>PHP (+12.51%)</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>+2.95%</t>
+          <t>+4.96%</t>
         </is>
       </c>
     </row>

</xml_diff>